<commit_message>
feat(trabajadores): escolaridad y estado civil opcionales
- Formulario: sin asterisco ni regla de obligatorio; opción
  "-Sin especificar-" para dejar el campo vacío o borrarlo.
- Tabla de trabajadores: muestra "-" cuando no hay dato.
- Visualizadores de nota médica y nota aclaratoria: la frase de
  escolaridad / estado civil solo aparece si hay dato.
- Plantillas de importación regeneradas (columnas marcadas OPCIONAL) y
  README actualizado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template/Plantilla Importar Trabajadores.xlsx
+++ b/public/template/Plantilla Importar Trabajadores.xlsx
@@ -1,180 +1,171 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_57560D40E59FE63C073329A7A4CEBB016EC991B1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB7B1DB3-1FCB-42C2-8A6A-9E4A3AF8E4D3}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Datos" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Datos" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF666666"/>
-            <rFont val="Calibri"/>
-          </rPr>
-          <t>OPCIONAL
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <color rgb="FF666666"/>
+            <sz val="9"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">OPCIONAL
 Número de empleado (1-7 dígitos).</t>
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF666666"/>
-            <rFont val="Calibri"/>
-          </rPr>
-          <t>OPCIONAL
+    <comment ref="B1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <color rgb="FF666666"/>
+            <sz val="9"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">OPCIONAL
 Identificador de seguridad social (4-30 caracteres).</t>
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF666666"/>
+    <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <color rgb="FF666666"/>
+            <sz val="9"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t>OPCIONAL</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <color rgb="FF666666"/>
+            <sz val="9"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t>OPCIONAL (requiere primerApellido)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <color rgb="FF666666"/>
+            <sz val="9"/>
             <rFont val="Calibri"/>
           </rPr>
           <t>OBLIGATORIO</t>
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF666666"/>
-            <rFont val="Calibri"/>
-          </rPr>
-          <t>OPCIONAL</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF666666"/>
-            <rFont val="Calibri"/>
-          </rPr>
-          <t>OBLIGATORIO</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF666666"/>
-            <rFont val="Calibri"/>
-          </rPr>
-          <t>OBLIGATORIO
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <color rgb="FF666666"/>
+            <sz val="9"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">OBLIGATORIO
 Formato fecha (YYYY-MM-DD o fecha de Excel).
 Edad permitida: 18-70 años.</t>
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF666666"/>
-            <rFont val="Calibri"/>
-          </rPr>
-          <t>OBLIGATORIO
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <color rgb="FF666666"/>
+            <sz val="9"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">OBLIGATORIO
 Masculino, Femenino o Intersexual.</t>
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF666666"/>
-            <rFont val="Calibri"/>
-          </rPr>
-          <t>OBLIGATORIO
+    <comment ref="H1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <color rgb="FF666666"/>
+            <sz val="9"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">OPCIONAL
 Primaria, Secundaria, Preparatoria, Licenciatura, Maestría, Doctorado o Nula.</t>
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF666666"/>
+    <comment ref="I1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <color rgb="FF666666"/>
+            <sz val="9"/>
             <rFont val="Calibri"/>
           </rPr>
           <t>OBLIGATORIO</t>
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF666666"/>
-            <rFont val="Calibri"/>
-          </rPr>
-          <t>OPCIONAL
+    <comment ref="J1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <color rgb="FF666666"/>
+            <sz val="9"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">OPCIONAL
 Fecha estimada de ingreso.
 Si no se conoce la exacta, usar el día 1 del mes más cercano.</t>
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF666666"/>
-            <rFont val="Calibri"/>
-          </rPr>
-          <t>OPCIONAL
+    <comment ref="K1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <color rgb="FF666666"/>
+            <sz val="9"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">OPCIONAL
 10 dígitos (México).</t>
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF666666"/>
-            <rFont val="Calibri"/>
-          </rPr>
-          <t>OBLIGATORIO
+    <comment ref="L1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <color rgb="FF666666"/>
+            <sz val="9"/>
+            <rFont val="Calibri"/>
+          </rPr>
+          <t xml:space="preserve">OPCIONAL
 Soltero/a, Casado/a, Unión libre, Separado/a, Divorciado/a o Viudo/a.</t>
         </r>
       </text>
@@ -184,7 +175,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>numeroEmpleado</t>
   </si>
@@ -220,6 +211,9 @@
   </si>
   <si>
     <t>estadoCivil</t>
+  </si>
+  <si>
+    <t>1001</t>
   </si>
   <si>
     <t>GARCIA</t>
@@ -249,23 +243,18 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF666666"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -636,9 +625,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -688,40 +677,43 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" s="2">
         <v>33008</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J2" s="2">
         <v>45292</v>
       </c>
       <c r="K2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>